<commit_message>
feat(route-pricing): migrate bảng giá CLF thành công
Chuẩn hóa dấu thanh địa danh, seed CLF theo price_book và cascade kỳ điều chỉnh.
</commit_message>
<xml_diff>
--- a/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
+++ b/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\web_app_phuphatcorp\reference\xu_ly_du_lieu_ke_toan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881999CD-983D-47C3-9CD0-81A1476630C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B90B21-E6F0-446A-9758-2ED2C57165B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="662">
   <si>
     <t>STT</t>
   </si>
@@ -1989,9 +1989,6 @@
     <t>Bà Rịa, Phú Mỹ, Tân Phước , Châu Pha , Hồ Tràm , Long Điền, Ngãi Giao</t>
   </si>
   <si>
-    <t>Bến Cát, Hòa Lợi, Hòa Phú, Long Nguyên, Mỹ Phước, Tân Hiệp, Tân Khánh, Tân Uyên, Tây Nam, Thới Hòa, Vĩnh Tân, Bắc Tân Uyên</t>
-  </si>
-  <si>
     <t>Wincom Bình dương</t>
   </si>
   <si>
@@ -2010,15 +2007,9 @@
     <t>Bảo Lộc , B'Lao</t>
   </si>
   <si>
-    <t>Đức Trọng, Hiệp Thạnh, Phú Hội</t>
-  </si>
-  <si>
     <t>Hàm Thắng, Phú Thủy, Tuyên Quang, Lương Sơn</t>
   </si>
   <si>
-    <t>Lâm Viên-Đà Lạt, Xuân Hương-Đà Lạt, Đơn Dương</t>
-  </si>
-  <si>
     <t>Đăk Cấm, Kon Tum, Bờ Y</t>
   </si>
   <si>
@@ -2028,9 +2019,6 @@
     <t>Khánh Hậu, Long An, Tân An, Bến Lức, Bình Đức, Đức Hòa, Đức Lập, Hậu Nghĩa, Hòa Khánh, Long Cang, Mỹ Hạnh, Mỹ Yên, Rạch Kiến , Tân Lân</t>
   </si>
   <si>
-    <t>NPP Mộc Hóa</t>
-  </si>
-  <si>
     <t>Long Đức, Nguyệt Hóa , Trà Vinh</t>
   </si>
   <si>
@@ -2077,6 +2065,15 @@
   </si>
   <si>
     <t>Bàu Bàng, Long Hòa, Phước Hòa</t>
+  </si>
+  <si>
+    <t>Bến Cát, Hòa Lợi, Long Nguyên, Tân Hiệp, Tân Khánh, Tân Uyên, Tây Nam, Thới Hòa, Vĩnh Tân, Bắc Tân Uyên</t>
+  </si>
+  <si>
+    <t>Đức Trọng, Hiệp Thạnh</t>
+  </si>
+  <si>
+    <t>Lâm Viên - Đà Lạt, Xuân Hương - Đà Lạt, Đơn Dương</t>
   </si>
 </sst>
 </file>
@@ -6228,19 +6225,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A247:G247"/>
-    <mergeCell ref="A170:G170"/>
-    <mergeCell ref="A183:G183"/>
-    <mergeCell ref="A234:G234"/>
-    <mergeCell ref="A221:G221"/>
-    <mergeCell ref="A208:G208"/>
-    <mergeCell ref="A195:G195"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A49:G49"/>
     <mergeCell ref="A109:G109"/>
     <mergeCell ref="A97:G97"/>
     <mergeCell ref="A85:G85"/>
@@ -6249,6 +6233,19 @@
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A145:G145"/>
     <mergeCell ref="A121:G121"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A247:G247"/>
+    <mergeCell ref="A170:G170"/>
+    <mergeCell ref="A183:G183"/>
+    <mergeCell ref="A234:G234"/>
+    <mergeCell ref="A221:G221"/>
+    <mergeCell ref="A208:G208"/>
+    <mergeCell ref="A195:G195"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26433,10 +26430,10 @@
         <v>608</v>
       </c>
       <c r="D2" s="124" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="E2" s="124" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>2</v>
@@ -26568,7 +26565,7 @@
         <v>302000</v>
       </c>
       <c r="K4" s="11">
-        <v>543000</v>
+        <v>522000</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
@@ -26629,7 +26626,7 @@
         <v>452000</v>
       </c>
       <c r="K5" s="11">
-        <v>711000</v>
+        <v>684000</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -26690,7 +26687,7 @@
         <v>372000</v>
       </c>
       <c r="K6" s="11">
-        <v>606000</v>
+        <v>583000</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -26810,7 +26807,7 @@
         <v>402000</v>
       </c>
       <c r="K8" s="11">
-        <v>648000</v>
+        <v>623000</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -26871,7 +26868,7 @@
         <v>443000</v>
       </c>
       <c r="K9" s="11">
-        <v>752000</v>
+        <v>723000</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
@@ -26932,7 +26929,7 @@
         <v>422000</v>
       </c>
       <c r="K10" s="11">
-        <v>679000</v>
+        <v>653000</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -26993,7 +26990,7 @@
         <v>503000</v>
       </c>
       <c r="K11" s="11">
-        <v>784000</v>
+        <v>754000</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -27054,7 +27051,7 @@
         <v>302000</v>
       </c>
       <c r="K12" s="11">
-        <v>502000</v>
+        <v>483000</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
@@ -27115,7 +27112,7 @@
         <v>352000</v>
       </c>
       <c r="K13" s="11">
-        <v>575000</v>
+        <v>553000</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -27176,7 +27173,7 @@
         <v>382000</v>
       </c>
       <c r="K14" s="11">
-        <v>564000</v>
+        <v>543000</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -27237,7 +27234,7 @@
         <v>321000</v>
       </c>
       <c r="K15" s="11">
-        <v>575000</v>
+        <v>553000</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
@@ -27298,7 +27295,7 @@
         <v>355000</v>
       </c>
       <c r="K16" s="11">
-        <v>512000</v>
+        <v>493000</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
@@ -27654,7 +27651,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="11">
-        <v>428000</v>
+        <v>412000</v>
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -27715,7 +27712,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="11">
-        <v>575000</v>
+        <v>553000</v>
       </c>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -27776,7 +27773,7 @@
         <v>342000</v>
       </c>
       <c r="K24" s="11">
-        <v>502000</v>
+        <v>483000</v>
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -27837,7 +27834,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="11">
-        <v>314000</v>
+        <v>302000</v>
       </c>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
@@ -27898,7 +27895,7 @@
         <v>342000</v>
       </c>
       <c r="K26" s="11">
-        <v>523000</v>
+        <v>503000</v>
       </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -27959,7 +27956,7 @@
         <v>352000</v>
       </c>
       <c r="K27" s="11">
-        <v>491000</v>
+        <v>472000</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -28020,7 +28017,7 @@
         <v>302000</v>
       </c>
       <c r="K28" s="11">
-        <v>491000</v>
+        <v>472000</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -28081,7 +28078,7 @@
         <v>342000</v>
       </c>
       <c r="K29" s="11">
-        <v>481000</v>
+        <v>463000</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -28142,7 +28139,7 @@
         <v>302000</v>
       </c>
       <c r="K30" s="11">
-        <v>428000</v>
+        <v>412000</v>
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -28419,7 +28416,7 @@
         <v>83</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="D35" s="114"/>
       <c r="E35" s="114"/>
@@ -28475,7 +28472,7 @@
         <v>33</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>631</v>
@@ -28498,7 +28495,7 @@
         <v>0</v>
       </c>
       <c r="K36" s="11">
-        <v>366000</v>
+        <v>352000</v>
       </c>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -28536,7 +28533,7 @@
         <v>34</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>632</v>
@@ -28559,7 +28556,7 @@
         <v>0</v>
       </c>
       <c r="K37" s="11">
-        <v>408000</v>
+        <v>392000</v>
       </c>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -28597,10 +28594,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="D38" s="114"/>
       <c r="E38" s="114"/>
@@ -28620,7 +28617,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="11">
-        <v>428000</v>
+        <v>412000</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -28658,10 +28655,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>633</v>
+        <v>659</v>
       </c>
       <c r="D39" s="114"/>
       <c r="E39" s="114"/>
@@ -28681,7 +28678,7 @@
         <v>0</v>
       </c>
       <c r="K39" s="11">
-        <v>408000</v>
+        <v>392000</v>
       </c>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -28716,12 +28713,12 @@
     <row r="40" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="B40" s="15" t="s">
-        <v>650</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>634</v>
-      </c>
-      <c r="D40" s="114"/>
+        <v>646</v>
+      </c>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15" t="s">
+        <v>633</v>
+      </c>
       <c r="E40" s="114"/>
       <c r="F40" s="11">
         <v>1328000</v>
@@ -28734,7 +28731,9 @@
         <v>302000</v>
       </c>
       <c r="J40" s="11"/>
-      <c r="K40" s="11"/>
+      <c r="K40" s="11">
+        <v>392000</v>
+      </c>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
@@ -28771,10 +28770,10 @@
         <v>37</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D41" s="114"/>
       <c r="E41" s="114"/>
@@ -28794,7 +28793,7 @@
         <v>266000</v>
       </c>
       <c r="K41" s="11">
-        <v>314000</v>
+        <v>302000</v>
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -28832,7 +28831,7 @@
         <v>38</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>89</v>
@@ -28857,7 +28856,7 @@
         <v>291000</v>
       </c>
       <c r="K42" s="11">
-        <v>366000</v>
+        <v>352000</v>
       </c>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -28895,7 +28894,7 @@
         <v>39</v>
       </c>
       <c r="B43" s="117" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C43" s="15"/>
       <c r="D43" s="114" t="s">
@@ -28954,10 +28953,10 @@
         <v>40</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D44" s="114"/>
       <c r="E44" s="114"/>
@@ -28977,7 +28976,7 @@
         <v>0</v>
       </c>
       <c r="K44" s="11">
-        <v>428000</v>
+        <v>412000</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -29097,7 +29096,7 @@
         <v>623000</v>
       </c>
       <c r="K46" s="11">
-        <v>888000</v>
+        <v>854000</v>
       </c>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -29138,7 +29137,7 @@
         <v>33</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D47" s="114"/>
       <c r="E47" s="114"/>
@@ -29197,7 +29196,7 @@
         <v>33</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D48" s="114"/>
       <c r="E48" s="114"/>
@@ -29217,7 +29216,7 @@
         <v>533000</v>
       </c>
       <c r="K48" s="11">
-        <v>878000</v>
+        <v>845000</v>
       </c>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -29317,7 +29316,7 @@
         <v>94</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D50" s="114"/>
       <c r="E50" s="114"/>
@@ -29337,7 +29336,7 @@
         <v>402000</v>
       </c>
       <c r="K50" s="11">
-        <v>627000</v>
+        <v>603000</v>
       </c>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -29437,7 +29436,7 @@
         <v>94</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>640</v>
+        <v>660</v>
       </c>
       <c r="D52" s="114"/>
       <c r="E52" s="114"/>
@@ -29457,7 +29456,7 @@
         <v>483000</v>
       </c>
       <c r="K52" s="11">
-        <v>732000</v>
+        <v>704000</v>
       </c>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
@@ -29498,7 +29497,7 @@
         <v>94</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D53" s="114"/>
       <c r="E53" s="114"/>
@@ -29518,7 +29517,7 @@
         <v>0</v>
       </c>
       <c r="K53" s="11">
-        <v>575000</v>
+        <v>553000</v>
       </c>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
@@ -29579,7 +29578,7 @@
         <v>0</v>
       </c>
       <c r="K54" s="11">
-        <v>543000</v>
+        <v>522000</v>
       </c>
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
@@ -29620,7 +29619,7 @@
         <v>94</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>642</v>
+        <v>661</v>
       </c>
       <c r="D55" s="114"/>
       <c r="E55" s="114"/>
@@ -29640,7 +29639,7 @@
         <v>513000</v>
       </c>
       <c r="K55" s="11">
-        <v>773000</v>
+        <v>744000</v>
       </c>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
@@ -29701,7 +29700,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="11">
-        <v>711000</v>
+        <v>684000</v>
       </c>
       <c r="L56" s="1"/>
       <c r="M56" s="1"/>
@@ -29801,7 +29800,7 @@
         <v>13</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="D58" s="114"/>
       <c r="E58" s="114"/>
@@ -29939,7 +29938,7 @@
         <v>0</v>
       </c>
       <c r="K60" s="11">
-        <v>491000</v>
+        <v>472000</v>
       </c>
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
@@ -29980,7 +29979,7 @@
         <v>9</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="D61" s="114"/>
       <c r="E61" s="114"/>
@@ -30000,7 +29999,7 @@
         <v>0</v>
       </c>
       <c r="K61" s="11">
-        <v>491000</v>
+        <v>472000</v>
       </c>
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
@@ -30100,7 +30099,7 @@
         <v>9</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="D63" s="114"/>
       <c r="E63" s="114"/>
@@ -30120,7 +30119,7 @@
         <v>251000</v>
       </c>
       <c r="K63" s="11">
-        <v>334000</v>
+        <v>321000</v>
       </c>
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
@@ -30161,7 +30160,7 @@
         <v>9</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>646</v>
+        <v>99</v>
       </c>
       <c r="D64" s="114"/>
       <c r="E64" s="114"/>
@@ -30217,7 +30216,7 @@
         <v>61</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C65" s="15" t="s">
         <v>609</v>
@@ -30240,7 +30239,7 @@
         <v>221000</v>
       </c>
       <c r="K65" s="11">
-        <v>272000</v>
+        <v>262000</v>
       </c>
       <c r="L65" s="1"/>
       <c r="M65" s="1"/>
@@ -30278,7 +30277,7 @@
         <v>62</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C66" s="15" t="s">
         <v>609</v>
@@ -30303,7 +30302,7 @@
         <v>271000</v>
       </c>
       <c r="K66" s="11">
-        <v>355000</v>
+        <v>342000</v>
       </c>
       <c r="L66" s="1"/>
       <c r="M66" s="1"/>
@@ -30364,7 +30363,7 @@
         <v>321000</v>
       </c>
       <c r="K67" s="11">
-        <v>502000</v>
+        <v>483000</v>
       </c>
       <c r="L67" s="1"/>
       <c r="M67" s="1"/>
@@ -30405,7 +30404,7 @@
         <v>19</v>
       </c>
       <c r="C68" s="116" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="D68" s="114"/>
       <c r="E68" s="114"/>
@@ -30425,7 +30424,7 @@
         <v>352000</v>
       </c>
       <c r="K68" s="11">
-        <v>575000</v>
+        <v>553000</v>
       </c>
       <c r="L68" s="1"/>
       <c r="M68" s="1"/>
@@ -30466,7 +30465,7 @@
         <v>19</v>
       </c>
       <c r="C69" s="115" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="D69" s="114"/>
       <c r="E69" s="114"/>
@@ -30486,7 +30485,7 @@
         <v>282000</v>
       </c>
       <c r="K69" s="11">
-        <v>481000</v>
+        <v>463000</v>
       </c>
       <c r="L69" s="1"/>
       <c r="M69" s="1"/>
@@ -30558,10 +30557,10 @@
         <v>607</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="E73" s="17" t="s">
         <v>6</v>
@@ -30594,10 +30593,10 @@
         <v>1</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="D74" s="15"/>
       <c r="E74" s="8">
@@ -30632,13 +30631,13 @@
         <v>2</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C75" s="15" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="D75" s="16" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="E75" s="14">
         <v>221000</v>
@@ -30672,13 +30671,13 @@
         <v>3</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="D76" s="16" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="E76" s="14">
         <v>181000</v>
@@ -30712,13 +30711,13 @@
         <v>4</v>
       </c>
       <c r="B77" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>655</v>
+      </c>
+      <c r="D77" s="43" t="s">
         <v>650</v>
-      </c>
-      <c r="C77" s="15" t="s">
-        <v>659</v>
-      </c>
-      <c r="D77" s="43" t="s">
-        <v>654</v>
       </c>
       <c r="E77" s="44">
         <v>625000</v>
@@ -30752,13 +30751,13 @@
         <v>5</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="D78" s="43" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="E78" s="44">
         <v>529000</v>
@@ -30841,7 +30840,7 @@
         <v>607</v>
       </c>
       <c r="D83" s="120" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="E83" s="17" t="s">
         <v>24</v>
@@ -30945,7 +30944,7 @@
         <v>70</v>
       </c>
       <c r="D85" s="19" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="E85" s="20">
         <v>522000</v>

</xml_diff>

<commit_message>
feat(route-pricing): seed VP-hiep phuoc (f) và cascade nhãn by_truck
</commit_message>
<xml_diff>
--- a/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
+++ b/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\web_app_phuphatcorp\reference\xu_ly_du_lieu_ke_toan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4C4D34-CFB4-4C9D-9F49-4151C2EFCBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B917FD6-BEE5-45C1-A4B0-0B4318A1E90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TINH GIA DAU" sheetId="36" r:id="rId1"/>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3086" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3088" uniqueCount="710">
   <si>
     <t>STT</t>
   </si>
@@ -2241,6 +2241,9 @@
   </si>
   <si>
     <t>Ayun Pa</t>
+  </si>
+  <si>
+    <t>Skip</t>
   </si>
   <si>
     <t>Skip - Giống Lâm Đồng - Hiệp Thạnh</t>
@@ -53189,7 +53192,9 @@
         <v>375</v>
       </c>
       <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
+      <c r="E23" s="21" t="s">
+        <v>706</v>
+      </c>
       <c r="F23" s="56">
         <v>0</v>
       </c>
@@ -58349,11 +58354,11 @@
       <c r="B114" s="51" t="s">
         <v>638</v>
       </c>
-      <c r="C114" s="50" t="s">
+      <c r="C114" s="50"/>
+      <c r="D114" s="50"/>
+      <c r="E114" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="D114" s="50"/>
-      <c r="E114" s="50"/>
       <c r="F114" s="58">
         <v>0</v>
       </c>
@@ -58525,7 +58530,7 @@
       </c>
       <c r="D117" s="50"/>
       <c r="E117" s="50" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F117" s="58">
         <v>1328000</v>
@@ -58869,7 +58874,7 @@
       </c>
       <c r="D123" s="50"/>
       <c r="E123" s="50" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F123" s="58">
         <v>1328000</v>
@@ -59839,7 +59844,9 @@
         <v>461</v>
       </c>
       <c r="D140" s="50"/>
-      <c r="E140" s="50"/>
+      <c r="E140" s="50" t="s">
+        <v>706</v>
+      </c>
       <c r="F140" s="58">
         <v>0</v>
       </c>
@@ -60690,9 +60697,7 @@
       <c r="B155" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="C155" s="50" t="s">
-        <v>95</v>
-      </c>
+      <c r="C155" s="50"/>
       <c r="D155" s="50"/>
       <c r="E155" s="50"/>
       <c r="F155" s="58">
@@ -61265,7 +61270,7 @@
       </c>
       <c r="D165" s="50"/>
       <c r="E165" s="50" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="F165" s="58">
         <v>0</v>
@@ -62577,7 +62582,9 @@
         <v>320</v>
       </c>
       <c r="D188" s="50"/>
-      <c r="E188" s="50"/>
+      <c r="E188" s="50" t="s">
+        <v>706</v>
+      </c>
       <c r="F188" s="58">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
chore: cập nhật note Skip trên sheet VP-hiep phuoc (f)
</commit_message>
<xml_diff>
--- a/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
+++ b/reference/xu_ly_du_lieu_ke_toan/BẢNG GIÁ - 2026 - 1.8.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\web_app_phuphatcorp\reference\xu_ly_du_lieu_ke_toan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4C4D34-CFB4-4C9D-9F49-4151C2EFCBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B917FD6-BEE5-45C1-A4B0-0B4318A1E90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TINH GIA DAU" sheetId="36" r:id="rId1"/>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3086" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3088" uniqueCount="710">
   <si>
     <t>STT</t>
   </si>
@@ -2241,6 +2241,9 @@
   </si>
   <si>
     <t>Ayun Pa</t>
+  </si>
+  <si>
+    <t>Skip</t>
   </si>
   <si>
     <t>Skip - Giống Lâm Đồng - Hiệp Thạnh</t>
@@ -53189,7 +53192,9 @@
         <v>375</v>
       </c>
       <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
+      <c r="E23" s="21" t="s">
+        <v>706</v>
+      </c>
       <c r="F23" s="56">
         <v>0</v>
       </c>
@@ -58349,11 +58354,11 @@
       <c r="B114" s="51" t="s">
         <v>638</v>
       </c>
-      <c r="C114" s="50" t="s">
+      <c r="C114" s="50"/>
+      <c r="D114" s="50"/>
+      <c r="E114" s="50" t="s">
         <v>366</v>
       </c>
-      <c r="D114" s="50"/>
-      <c r="E114" s="50"/>
       <c r="F114" s="58">
         <v>0</v>
       </c>
@@ -58525,7 +58530,7 @@
       </c>
       <c r="D117" s="50"/>
       <c r="E117" s="50" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F117" s="58">
         <v>1328000</v>
@@ -58869,7 +58874,7 @@
       </c>
       <c r="D123" s="50"/>
       <c r="E123" s="50" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F123" s="58">
         <v>1328000</v>
@@ -59839,7 +59844,9 @@
         <v>461</v>
       </c>
       <c r="D140" s="50"/>
-      <c r="E140" s="50"/>
+      <c r="E140" s="50" t="s">
+        <v>706</v>
+      </c>
       <c r="F140" s="58">
         <v>0</v>
       </c>
@@ -60690,9 +60697,7 @@
       <c r="B155" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="C155" s="50" t="s">
-        <v>95</v>
-      </c>
+      <c r="C155" s="50"/>
       <c r="D155" s="50"/>
       <c r="E155" s="50"/>
       <c r="F155" s="58">
@@ -61265,7 +61270,7 @@
       </c>
       <c r="D165" s="50"/>
       <c r="E165" s="50" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="F165" s="58">
         <v>0</v>
@@ -62577,7 +62582,9 @@
         <v>320</v>
       </c>
       <c r="D188" s="50"/>
-      <c r="E188" s="50"/>
+      <c r="E188" s="50" t="s">
+        <v>706</v>
+      </c>
       <c r="F188" s="58">
         <v>0</v>
       </c>

</xml_diff>